<commit_message>
feat(rates): rate sheet carries Mode; add barge NLRTM-DEDUI card; migration 0013
gen_rate_sheet emits a Mode meta row per sheet + a BARGE NLRTM-DEDUI card (Low-Water
Surcharge); import_rate_sheet keys + writes rate_cards.mode; migration 0013 adds the column
(default FCL). Parser + round-trip tests cover the barge card (1x40HC = 755 EUR). xlsx regenerated.

Co-Authored-By: Claude Opus 4.8 (1M context) <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/rates/linkport-rate-sheet.xlsx
+++ b/rates/linkport-rate-sheet.xlsx
@@ -4,17 +4,24 @@
   <fileVersion appName="xl" lastEdited="5" lowestEdited="5" rupBuild="9303"/>
   <workbookPr defaultThemeVersion="164011" filterPrivacy="1"/>
   <sheets>
-    <sheet sheetId="1" name="NLRTM-USNYC" state="visible" r:id="rId4"/>
-    <sheet sheetId="2" name="NLRTM-USLAX" state="visible" r:id="rId5"/>
-    <sheet sheetId="3" name="DEHAM-USNYC" state="visible" r:id="rId6"/>
-    <sheet sheetId="4" name="About" state="visible" r:id="rId7"/>
+    <sheet sheetId="1" name="FCL NLRTM-USNYC" state="visible" r:id="rId4"/>
+    <sheet sheetId="2" name="FCL NLRTM-USLAX" state="visible" r:id="rId5"/>
+    <sheet sheetId="3" name="FCL DEHAM-USNYC" state="visible" r:id="rId6"/>
+    <sheet sheetId="4" name="BARGE NLRTM-DEDUI" state="visible" r:id="rId7"/>
+    <sheet sheetId="5" name="About" state="visible" r:id="rId8"/>
   </sheets>
   <calcPr calcId="171027"/>
 </workbook>
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="131" uniqueCount="38">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="171" uniqueCount="45">
+  <si>
+    <t>Mode</t>
+  </si>
+  <si>
+    <t>FCL</t>
+  </si>
   <si>
     <t>Lane</t>
   </si>
@@ -122,6 +129,21 @@
   </si>
   <si>
     <t>CONGESTION</t>
+  </si>
+  <si>
+    <t>BARGE</t>
+  </si>
+  <si>
+    <t>NLRTM-DEDUI</t>
+  </si>
+  <si>
+    <t>LWS</t>
+  </si>
+  <si>
+    <t>THC_RTM_BARGE</t>
+  </si>
+  <si>
+    <t>THC_DUI</t>
   </si>
   <si>
     <t>All figures are INVENTED placeholders — see docs/ASSUMPTIONS.md. Not real freight rates.</t>
@@ -508,7 +530,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <dimension ref="A1:E14"/>
+  <dimension ref="A1:E15"/>
   <sheetFormatPr defaultRowHeight="15" outlineLevelRow="0" outlineLevelCol="0" x14ac:dyDescent="55"/>
   <cols>
     <col min="1" max="5" width="24" customWidth="1"/>
@@ -538,43 +560,34 @@
         <v>5</v>
       </c>
     </row>
-    <row r="5" spans="1:5" s="1" customFormat="1" x14ac:dyDescent="0.25">
-      <c r="A5" s="1" t="s">
+    <row r="4" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A4" t="s">
         <v>6</v>
       </c>
-      <c r="B5" s="1" t="s">
+      <c r="B4" t="s">
         <v>7</v>
       </c>
-      <c r="C5" s="1" t="s">
+    </row>
+    <row r="6" spans="1:5" s="1" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A6" s="1" t="s">
         <v>8</v>
       </c>
-      <c r="D5" s="1" t="s">
+      <c r="B6" s="1" t="s">
         <v>9</v>
       </c>
-      <c r="E5" s="1" t="s">
+      <c r="C6" s="1" t="s">
         <v>10</v>
       </c>
-    </row>
-    <row r="6" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A6" t="s">
+      <c r="D6" s="1" t="s">
         <v>11</v>
       </c>
-      <c r="B6" t="s">
+      <c r="E6" s="1" t="s">
         <v>12</v>
-      </c>
-      <c r="C6" t="s">
-        <v>13</v>
-      </c>
-      <c r="D6">
-        <v>1800</v>
-      </c>
-      <c r="E6">
-        <v>0</v>
       </c>
     </row>
     <row r="7" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A7" t="s">
-        <v>11</v>
+        <v>13</v>
       </c>
       <c r="B7" t="s">
         <v>14</v>
@@ -583,15 +596,15 @@
         <v>15</v>
       </c>
       <c r="D7">
-        <v>2400</v>
+        <v>1800</v>
       </c>
       <c r="E7">
-        <v>1</v>
+        <v>0</v>
       </c>
     </row>
     <row r="8" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A8" t="s">
-        <v>11</v>
+        <v>13</v>
       </c>
       <c r="B8" t="s">
         <v>16</v>
@@ -600,111 +613,128 @@
         <v>17</v>
       </c>
       <c r="D8">
-        <v>2550</v>
+        <v>2400</v>
       </c>
       <c r="E8">
-        <v>2</v>
+        <v>1</v>
       </c>
     </row>
     <row r="9" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A9" t="s">
+        <v>13</v>
+      </c>
+      <c r="B9" t="s">
         <v>18</v>
       </c>
-      <c r="B9" t="s">
+      <c r="C9" t="s">
         <v>19</v>
       </c>
-      <c r="C9" t="s">
-        <v>20</v>
-      </c>
       <c r="D9">
-        <v>320</v>
+        <v>2550</v>
       </c>
       <c r="E9">
-        <v>0</v>
+        <v>2</v>
       </c>
     </row>
     <row r="10" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A10" t="s">
-        <v>18</v>
+        <v>20</v>
       </c>
       <c r="B10" t="s">
         <v>21</v>
       </c>
       <c r="C10" t="s">
-        <v>20</v>
+        <v>22</v>
       </c>
       <c r="D10">
-        <v>225</v>
+        <v>320</v>
       </c>
       <c r="E10">
-        <v>1</v>
+        <v>0</v>
       </c>
     </row>
     <row r="11" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A11" t="s">
-        <v>18</v>
+        <v>20</v>
       </c>
       <c r="B11" t="s">
-        <v>22</v>
+        <v>23</v>
       </c>
       <c r="C11" t="s">
-        <v>20</v>
+        <v>22</v>
       </c>
       <c r="D11">
-        <v>290</v>
+        <v>225</v>
       </c>
       <c r="E11">
-        <v>2</v>
+        <v>1</v>
       </c>
     </row>
     <row r="12" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A12" t="s">
-        <v>18</v>
+        <v>20</v>
       </c>
       <c r="B12" t="s">
-        <v>23</v>
+        <v>24</v>
       </c>
       <c r="C12" t="s">
-        <v>20</v>
+        <v>22</v>
       </c>
       <c r="D12">
-        <v>25</v>
+        <v>290</v>
       </c>
       <c r="E12">
-        <v>3</v>
+        <v>2</v>
       </c>
     </row>
     <row r="13" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A13" t="s">
-        <v>24</v>
+        <v>20</v>
       </c>
       <c r="B13" t="s">
         <v>25</v>
       </c>
       <c r="C13" t="s">
-        <v>20</v>
+        <v>22</v>
       </c>
       <c r="D13">
-        <v>65</v>
+        <v>25</v>
       </c>
       <c r="E13">
-        <v>0</v>
+        <v>3</v>
       </c>
     </row>
     <row r="14" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A14" t="s">
-        <v>24</v>
+        <v>26</v>
       </c>
       <c r="B14" t="s">
+        <v>27</v>
+      </c>
+      <c r="C14" t="s">
+        <v>22</v>
+      </c>
+      <c r="D14">
+        <v>65</v>
+      </c>
+      <c r="E14">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="15" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A15" t="s">
         <v>26</v>
       </c>
-      <c r="C14" t="s">
-        <v>20</v>
-      </c>
-      <c r="D14">
+      <c r="B15" t="s">
+        <v>28</v>
+      </c>
+      <c r="C15" t="s">
+        <v>22</v>
+      </c>
+      <c r="D15">
         <v>45</v>
       </c>
-      <c r="E14">
+      <c r="E15">
         <v>1</v>
       </c>
     </row>
@@ -715,6 +745,273 @@
 </file>
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
+  <dimension ref="A1:E18"/>
+  <sheetFormatPr defaultRowHeight="15" outlineLevelRow="0" outlineLevelCol="0" x14ac:dyDescent="55"/>
+  <cols>
+    <col min="1" max="5" width="24" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A1" t="s">
+        <v>0</v>
+      </c>
+      <c r="B1" t="s">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="2" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A2" t="s">
+        <v>2</v>
+      </c>
+      <c r="B2" t="s">
+        <v>29</v>
+      </c>
+    </row>
+    <row r="3" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A3" t="s">
+        <v>4</v>
+      </c>
+      <c r="B3" t="s">
+        <v>5</v>
+      </c>
+    </row>
+    <row r="4" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A4" t="s">
+        <v>6</v>
+      </c>
+      <c r="B4" t="s">
+        <v>7</v>
+      </c>
+    </row>
+    <row r="6" spans="1:5" s="1" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A6" s="1" t="s">
+        <v>8</v>
+      </c>
+      <c r="B6" s="1" t="s">
+        <v>9</v>
+      </c>
+      <c r="C6" s="1" t="s">
+        <v>10</v>
+      </c>
+      <c r="D6" s="1" t="s">
+        <v>11</v>
+      </c>
+      <c r="E6" s="1" t="s">
+        <v>12</v>
+      </c>
+    </row>
+    <row r="7" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A7" t="s">
+        <v>13</v>
+      </c>
+      <c r="B7" t="s">
+        <v>14</v>
+      </c>
+      <c r="C7" t="s">
+        <v>15</v>
+      </c>
+      <c r="D7">
+        <v>2200</v>
+      </c>
+      <c r="E7">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="8" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A8" t="s">
+        <v>13</v>
+      </c>
+      <c r="B8" t="s">
+        <v>16</v>
+      </c>
+      <c r="C8" t="s">
+        <v>17</v>
+      </c>
+      <c r="D8">
+        <v>2900</v>
+      </c>
+      <c r="E8">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="9" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A9" t="s">
+        <v>13</v>
+      </c>
+      <c r="B9" t="s">
+        <v>18</v>
+      </c>
+      <c r="C9" t="s">
+        <v>19</v>
+      </c>
+      <c r="D9">
+        <v>3050</v>
+      </c>
+      <c r="E9">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="10" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A10" t="s">
+        <v>13</v>
+      </c>
+      <c r="B10" t="s">
+        <v>30</v>
+      </c>
+      <c r="C10" t="s">
+        <v>31</v>
+      </c>
+      <c r="D10">
+        <v>3250</v>
+      </c>
+      <c r="E10">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="11" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A11" t="s">
+        <v>20</v>
+      </c>
+      <c r="B11" t="s">
+        <v>21</v>
+      </c>
+      <c r="C11" t="s">
+        <v>22</v>
+      </c>
+      <c r="D11">
+        <v>360</v>
+      </c>
+      <c r="E11">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="12" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A12" t="s">
+        <v>20</v>
+      </c>
+      <c r="B12" t="s">
+        <v>32</v>
+      </c>
+      <c r="C12" t="s">
+        <v>22</v>
+      </c>
+      <c r="D12">
+        <v>140</v>
+      </c>
+      <c r="E12">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="13" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A13" t="s">
+        <v>20</v>
+      </c>
+      <c r="B13" t="s">
+        <v>23</v>
+      </c>
+      <c r="C13" t="s">
+        <v>22</v>
+      </c>
+      <c r="D13">
+        <v>225</v>
+      </c>
+      <c r="E13">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="14" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A14" t="s">
+        <v>20</v>
+      </c>
+      <c r="B14" t="s">
+        <v>33</v>
+      </c>
+      <c r="C14" t="s">
+        <v>22</v>
+      </c>
+      <c r="D14">
+        <v>310</v>
+      </c>
+      <c r="E14">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="15" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A15" t="s">
+        <v>20</v>
+      </c>
+      <c r="B15" t="s">
+        <v>25</v>
+      </c>
+      <c r="C15" t="s">
+        <v>22</v>
+      </c>
+      <c r="D15">
+        <v>25</v>
+      </c>
+      <c r="E15">
+        <v>4</v>
+      </c>
+    </row>
+    <row r="16" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A16" t="s">
+        <v>20</v>
+      </c>
+      <c r="B16" t="s">
+        <v>34</v>
+      </c>
+      <c r="C16" t="s">
+        <v>22</v>
+      </c>
+      <c r="D16">
+        <v>200</v>
+      </c>
+      <c r="E16">
+        <v>5</v>
+      </c>
+    </row>
+    <row r="17" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A17" t="s">
+        <v>26</v>
+      </c>
+      <c r="B17" t="s">
+        <v>27</v>
+      </c>
+      <c r="C17" t="s">
+        <v>22</v>
+      </c>
+      <c r="D17">
+        <v>65</v>
+      </c>
+      <c r="E17">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="18" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A18" t="s">
+        <v>26</v>
+      </c>
+      <c r="B18" t="s">
+        <v>28</v>
+      </c>
+      <c r="C18" t="s">
+        <v>22</v>
+      </c>
+      <c r="D18">
+        <v>45</v>
+      </c>
+      <c r="E18">
+        <v>1</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+  <pageSetup orientation="portrait" horizontalDpi="4294967295" verticalDpi="4294967295" scale="100" fitToWidth="1" fitToHeight="1"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
   <dimension ref="A1:E17"/>
   <sheetFormatPr defaultRowHeight="15" outlineLevelRow="0" outlineLevelCol="0" x14ac:dyDescent="55"/>
@@ -727,7 +1024,7 @@
         <v>0</v>
       </c>
       <c r="B1" t="s">
-        <v>27</v>
+        <v>1</v>
       </c>
     </row>
     <row r="2" spans="1:2" x14ac:dyDescent="0.25">
@@ -735,7 +1032,7 @@
         <v>2</v>
       </c>
       <c r="B2" t="s">
-        <v>3</v>
+        <v>35</v>
       </c>
     </row>
     <row r="3" spans="1:2" x14ac:dyDescent="0.25">
@@ -746,43 +1043,34 @@
         <v>5</v>
       </c>
     </row>
-    <row r="5" spans="1:5" s="1" customFormat="1" x14ac:dyDescent="0.25">
-      <c r="A5" s="1" t="s">
+    <row r="4" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A4" t="s">
         <v>6</v>
       </c>
-      <c r="B5" s="1" t="s">
+      <c r="B4" t="s">
         <v>7</v>
       </c>
-      <c r="C5" s="1" t="s">
+    </row>
+    <row r="6" spans="1:5" s="1" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A6" s="1" t="s">
         <v>8</v>
       </c>
-      <c r="D5" s="1" t="s">
+      <c r="B6" s="1" t="s">
         <v>9</v>
       </c>
-      <c r="E5" s="1" t="s">
+      <c r="C6" s="1" t="s">
         <v>10</v>
       </c>
-    </row>
-    <row r="6" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A6" t="s">
+      <c r="D6" s="1" t="s">
         <v>11</v>
       </c>
-      <c r="B6" t="s">
+      <c r="E6" s="1" t="s">
         <v>12</v>
-      </c>
-      <c r="C6" t="s">
-        <v>13</v>
-      </c>
-      <c r="D6">
-        <v>2200</v>
-      </c>
-      <c r="E6">
-        <v>0</v>
       </c>
     </row>
     <row r="7" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A7" t="s">
-        <v>11</v>
+        <v>13</v>
       </c>
       <c r="B7" t="s">
         <v>14</v>
@@ -791,15 +1079,15 @@
         <v>15</v>
       </c>
       <c r="D7">
-        <v>2900</v>
+        <v>1900</v>
       </c>
       <c r="E7">
-        <v>1</v>
+        <v>0</v>
       </c>
     </row>
     <row r="8" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A8" t="s">
-        <v>11</v>
+        <v>13</v>
       </c>
       <c r="B8" t="s">
         <v>16</v>
@@ -808,140 +1096,140 @@
         <v>17</v>
       </c>
       <c r="D8">
-        <v>3050</v>
+        <v>2500</v>
       </c>
       <c r="E8">
-        <v>2</v>
+        <v>1</v>
       </c>
     </row>
     <row r="9" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A9" t="s">
-        <v>11</v>
+        <v>13</v>
       </c>
       <c r="B9" t="s">
-        <v>28</v>
+        <v>18</v>
       </c>
       <c r="C9" t="s">
-        <v>29</v>
+        <v>19</v>
       </c>
       <c r="D9">
-        <v>3250</v>
+        <v>2650</v>
       </c>
       <c r="E9">
-        <v>3</v>
+        <v>2</v>
       </c>
     </row>
     <row r="10" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A10" t="s">
-        <v>18</v>
+        <v>13</v>
       </c>
       <c r="B10" t="s">
-        <v>19</v>
+        <v>30</v>
       </c>
       <c r="C10" t="s">
-        <v>20</v>
+        <v>31</v>
       </c>
       <c r="D10">
-        <v>360</v>
+        <v>2850</v>
       </c>
       <c r="E10">
-        <v>0</v>
+        <v>3</v>
       </c>
     </row>
     <row r="11" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A11" t="s">
-        <v>18</v>
+        <v>20</v>
       </c>
       <c r="B11" t="s">
-        <v>30</v>
+        <v>21</v>
       </c>
       <c r="C11" t="s">
-        <v>20</v>
+        <v>22</v>
       </c>
       <c r="D11">
-        <v>140</v>
+        <v>330</v>
       </c>
       <c r="E11">
-        <v>1</v>
+        <v>0</v>
       </c>
     </row>
     <row r="12" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A12" t="s">
-        <v>18</v>
+        <v>20</v>
       </c>
       <c r="B12" t="s">
-        <v>21</v>
+        <v>36</v>
       </c>
       <c r="C12" t="s">
-        <v>20</v>
+        <v>22</v>
       </c>
       <c r="D12">
-        <v>225</v>
+        <v>240</v>
       </c>
       <c r="E12">
-        <v>2</v>
+        <v>1</v>
       </c>
     </row>
     <row r="13" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A13" t="s">
-        <v>18</v>
+        <v>20</v>
       </c>
       <c r="B13" t="s">
-        <v>31</v>
+        <v>24</v>
       </c>
       <c r="C13" t="s">
-        <v>20</v>
+        <v>22</v>
       </c>
       <c r="D13">
-        <v>310</v>
+        <v>290</v>
       </c>
       <c r="E13">
-        <v>3</v>
+        <v>2</v>
       </c>
     </row>
     <row r="14" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A14" t="s">
-        <v>18</v>
+        <v>20</v>
       </c>
       <c r="B14" t="s">
-        <v>23</v>
+        <v>25</v>
       </c>
       <c r="C14" t="s">
-        <v>20</v>
+        <v>22</v>
       </c>
       <c r="D14">
         <v>25</v>
       </c>
       <c r="E14">
-        <v>4</v>
+        <v>3</v>
       </c>
     </row>
     <row r="15" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A15" t="s">
-        <v>18</v>
+        <v>20</v>
       </c>
       <c r="B15" t="s">
-        <v>32</v>
+        <v>37</v>
       </c>
       <c r="C15" t="s">
-        <v>20</v>
+        <v>22</v>
       </c>
       <c r="D15">
-        <v>200</v>
+        <v>175</v>
       </c>
       <c r="E15">
-        <v>5</v>
+        <v>4</v>
       </c>
     </row>
     <row r="16" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A16" t="s">
-        <v>24</v>
+        <v>26</v>
       </c>
       <c r="B16" t="s">
-        <v>25</v>
+        <v>27</v>
       </c>
       <c r="C16" t="s">
-        <v>20</v>
+        <v>22</v>
       </c>
       <c r="D16">
         <v>65</v>
@@ -952,260 +1240,18 @@
     </row>
     <row r="17" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A17" t="s">
-        <v>24</v>
+        <v>26</v>
       </c>
       <c r="B17" t="s">
-        <v>26</v>
+        <v>28</v>
       </c>
       <c r="C17" t="s">
-        <v>20</v>
+        <v>22</v>
       </c>
       <c r="D17">
         <v>45</v>
       </c>
       <c r="E17">
-        <v>1</v>
-      </c>
-    </row>
-  </sheetData>
-  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-  <pageSetup orientation="portrait" horizontalDpi="4294967295" verticalDpi="4294967295" scale="100" fitToWidth="1" fitToHeight="1"/>
-</worksheet>
-</file>
-
-<file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <dimension ref="A1:E16"/>
-  <sheetFormatPr defaultRowHeight="15" outlineLevelRow="0" outlineLevelCol="0" x14ac:dyDescent="55"/>
-  <cols>
-    <col min="1" max="5" width="24" customWidth="1"/>
-  </cols>
-  <sheetData>
-    <row r="1" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A1" t="s">
-        <v>0</v>
-      </c>
-      <c r="B1" t="s">
-        <v>33</v>
-      </c>
-    </row>
-    <row r="2" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A2" t="s">
-        <v>2</v>
-      </c>
-      <c r="B2" t="s">
-        <v>3</v>
-      </c>
-    </row>
-    <row r="3" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A3" t="s">
-        <v>4</v>
-      </c>
-      <c r="B3" t="s">
-        <v>5</v>
-      </c>
-    </row>
-    <row r="5" spans="1:5" s="1" customFormat="1" x14ac:dyDescent="0.25">
-      <c r="A5" s="1" t="s">
-        <v>6</v>
-      </c>
-      <c r="B5" s="1" t="s">
-        <v>7</v>
-      </c>
-      <c r="C5" s="1" t="s">
-        <v>8</v>
-      </c>
-      <c r="D5" s="1" t="s">
-        <v>9</v>
-      </c>
-      <c r="E5" s="1" t="s">
-        <v>10</v>
-      </c>
-    </row>
-    <row r="6" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A6" t="s">
-        <v>11</v>
-      </c>
-      <c r="B6" t="s">
-        <v>12</v>
-      </c>
-      <c r="C6" t="s">
-        <v>13</v>
-      </c>
-      <c r="D6">
-        <v>1900</v>
-      </c>
-      <c r="E6">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="7" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A7" t="s">
-        <v>11</v>
-      </c>
-      <c r="B7" t="s">
-        <v>14</v>
-      </c>
-      <c r="C7" t="s">
-        <v>15</v>
-      </c>
-      <c r="D7">
-        <v>2500</v>
-      </c>
-      <c r="E7">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="8" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A8" t="s">
-        <v>11</v>
-      </c>
-      <c r="B8" t="s">
-        <v>16</v>
-      </c>
-      <c r="C8" t="s">
-        <v>17</v>
-      </c>
-      <c r="D8">
-        <v>2650</v>
-      </c>
-      <c r="E8">
-        <v>2</v>
-      </c>
-    </row>
-    <row r="9" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A9" t="s">
-        <v>11</v>
-      </c>
-      <c r="B9" t="s">
-        <v>28</v>
-      </c>
-      <c r="C9" t="s">
-        <v>29</v>
-      </c>
-      <c r="D9">
-        <v>2850</v>
-      </c>
-      <c r="E9">
-        <v>3</v>
-      </c>
-    </row>
-    <row r="10" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A10" t="s">
-        <v>18</v>
-      </c>
-      <c r="B10" t="s">
-        <v>19</v>
-      </c>
-      <c r="C10" t="s">
-        <v>20</v>
-      </c>
-      <c r="D10">
-        <v>330</v>
-      </c>
-      <c r="E10">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="11" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A11" t="s">
-        <v>18</v>
-      </c>
-      <c r="B11" t="s">
-        <v>34</v>
-      </c>
-      <c r="C11" t="s">
-        <v>20</v>
-      </c>
-      <c r="D11">
-        <v>240</v>
-      </c>
-      <c r="E11">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="12" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A12" t="s">
-        <v>18</v>
-      </c>
-      <c r="B12" t="s">
-        <v>22</v>
-      </c>
-      <c r="C12" t="s">
-        <v>20</v>
-      </c>
-      <c r="D12">
-        <v>290</v>
-      </c>
-      <c r="E12">
-        <v>2</v>
-      </c>
-    </row>
-    <row r="13" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A13" t="s">
-        <v>18</v>
-      </c>
-      <c r="B13" t="s">
-        <v>23</v>
-      </c>
-      <c r="C13" t="s">
-        <v>20</v>
-      </c>
-      <c r="D13">
-        <v>25</v>
-      </c>
-      <c r="E13">
-        <v>3</v>
-      </c>
-    </row>
-    <row r="14" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A14" t="s">
-        <v>18</v>
-      </c>
-      <c r="B14" t="s">
-        <v>35</v>
-      </c>
-      <c r="C14" t="s">
-        <v>20</v>
-      </c>
-      <c r="D14">
-        <v>175</v>
-      </c>
-      <c r="E14">
-        <v>4</v>
-      </c>
-    </row>
-    <row r="15" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A15" t="s">
-        <v>24</v>
-      </c>
-      <c r="B15" t="s">
-        <v>25</v>
-      </c>
-      <c r="C15" t="s">
-        <v>20</v>
-      </c>
-      <c r="D15">
-        <v>65</v>
-      </c>
-      <c r="E15">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="16" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A16" t="s">
-        <v>24</v>
-      </c>
-      <c r="B16" t="s">
-        <v>26</v>
-      </c>
-      <c r="C16" t="s">
-        <v>20</v>
-      </c>
-      <c r="D16">
-        <v>45</v>
-      </c>
-      <c r="E16">
         <v>1</v>
       </c>
     </row>
@@ -1217,17 +1263,199 @@
 
 <file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
+  <dimension ref="A1:E13"/>
+  <sheetFormatPr defaultRowHeight="15" outlineLevelRow="0" outlineLevelCol="0" x14ac:dyDescent="55"/>
+  <cols>
+    <col min="1" max="5" width="24" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A1" t="s">
+        <v>0</v>
+      </c>
+      <c r="B1" t="s">
+        <v>38</v>
+      </c>
+    </row>
+    <row r="2" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A2" t="s">
+        <v>2</v>
+      </c>
+      <c r="B2" t="s">
+        <v>39</v>
+      </c>
+    </row>
+    <row r="3" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A3" t="s">
+        <v>4</v>
+      </c>
+      <c r="B3" t="s">
+        <v>5</v>
+      </c>
+    </row>
+    <row r="4" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A4" t="s">
+        <v>6</v>
+      </c>
+      <c r="B4" t="s">
+        <v>7</v>
+      </c>
+    </row>
+    <row r="6" spans="1:5" s="1" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A6" s="1" t="s">
+        <v>8</v>
+      </c>
+      <c r="B6" s="1" t="s">
+        <v>9</v>
+      </c>
+      <c r="C6" s="1" t="s">
+        <v>10</v>
+      </c>
+      <c r="D6" s="1" t="s">
+        <v>11</v>
+      </c>
+      <c r="E6" s="1" t="s">
+        <v>12</v>
+      </c>
+    </row>
+    <row r="7" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A7" t="s">
+        <v>13</v>
+      </c>
+      <c r="B7" t="s">
+        <v>14</v>
+      </c>
+      <c r="C7" t="s">
+        <v>15</v>
+      </c>
+      <c r="D7">
+        <v>280</v>
+      </c>
+      <c r="E7">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="8" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A8" t="s">
+        <v>13</v>
+      </c>
+      <c r="B8" t="s">
+        <v>16</v>
+      </c>
+      <c r="C8" t="s">
+        <v>17</v>
+      </c>
+      <c r="D8">
+        <v>420</v>
+      </c>
+      <c r="E8">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="9" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A9" t="s">
+        <v>13</v>
+      </c>
+      <c r="B9" t="s">
+        <v>18</v>
+      </c>
+      <c r="C9" t="s">
+        <v>19</v>
+      </c>
+      <c r="D9">
+        <v>420</v>
+      </c>
+      <c r="E9">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="10" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A10" t="s">
+        <v>20</v>
+      </c>
+      <c r="B10" t="s">
+        <v>40</v>
+      </c>
+      <c r="C10" t="s">
+        <v>22</v>
+      </c>
+      <c r="D10">
+        <v>95</v>
+      </c>
+      <c r="E10">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="11" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A11" t="s">
+        <v>20</v>
+      </c>
+      <c r="B11" t="s">
+        <v>41</v>
+      </c>
+      <c r="C11" t="s">
+        <v>22</v>
+      </c>
+      <c r="D11">
+        <v>95</v>
+      </c>
+      <c r="E11">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="12" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A12" t="s">
+        <v>20</v>
+      </c>
+      <c r="B12" t="s">
+        <v>42</v>
+      </c>
+      <c r="C12" t="s">
+        <v>22</v>
+      </c>
+      <c r="D12">
+        <v>110</v>
+      </c>
+      <c r="E12">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="13" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A13" t="s">
+        <v>26</v>
+      </c>
+      <c r="B13" t="s">
+        <v>27</v>
+      </c>
+      <c r="C13" t="s">
+        <v>22</v>
+      </c>
+      <c r="D13">
+        <v>35</v>
+      </c>
+      <c r="E13">
+        <v>0</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+  <pageSetup orientation="portrait" horizontalDpi="4294967295" verticalDpi="4294967295" scale="100" fitToWidth="1" fitToHeight="1"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
   <dimension ref="A1:A2"/>
   <sheetFormatPr defaultRowHeight="15" outlineLevelRow="0" outlineLevelCol="0" x14ac:dyDescent="55"/>
   <sheetData>
     <row r="1" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A1" t="s">
-        <v>36</v>
+        <v>43</v>
       </c>
     </row>
     <row r="2" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A2" t="s">
-        <v>37</v>
+        <v>44</v>
       </c>
     </row>
   </sheetData>

</xml_diff>